<commit_message>
Update example config xlsx
</commit_message>
<xml_diff>
--- a/config_examples/config_phase1_example.xlsx
+++ b/config_examples/config_phase1_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dinod\Desktop\EIS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u32r83\Desktop\EIS\config_examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289FB2FA-1035-4100-B86A-A9DCCEAC9C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6386DB2A-9930-48B7-8574-409EE7148A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -361,16 +361,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -390,7 +390,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>12.54</v>
       </c>
@@ -407,10 +407,10 @@
         <v>20</v>
       </c>
       <c r="F2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>19.899999999999999</v>
       </c>
@@ -427,10 +427,10 @@
         <v>20</v>
       </c>
       <c r="F3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>31.54</v>
       </c>
@@ -447,10 +447,10 @@
         <v>20</v>
       </c>
       <c r="F4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>49</v>
       </c>
@@ -467,10 +467,10 @@
         <v>20</v>
       </c>
       <c r="F5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>79.180000000000007</v>
       </c>
@@ -487,10 +487,10 @@
         <v>20</v>
       </c>
       <c r="F6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>125.79</v>
       </c>
@@ -507,10 +507,10 @@
         <v>20</v>
       </c>
       <c r="F7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>199.6</v>
       </c>
@@ -527,10 +527,10 @@
         <v>20</v>
       </c>
       <c r="F8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>314.45999999999998</v>
       </c>
@@ -547,10 +547,10 @@
         <v>20</v>
       </c>
       <c r="F9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>497.51</v>
       </c>
@@ -567,10 +567,10 @@
         <v>20</v>
       </c>
       <c r="F10">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>793.65</v>
       </c>
@@ -587,10 +587,10 @@
         <v>20</v>
       </c>
       <c r="F11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1234.57</v>
       </c>
@@ -607,10 +607,10 @@
         <v>20</v>
       </c>
       <c r="F12">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1960.78</v>
       </c>
@@ -627,10 +627,10 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3030.3</v>
       </c>
@@ -647,10 +647,10 @@
         <v>20</v>
       </c>
       <c r="F14">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4761.91</v>
       </c>
@@ -667,7 +667,7 @@
         <v>20</v>
       </c>
       <c r="F15">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>